<commit_message>
Agenda Agenda: Calendário, validação de horários e upload de estoque - Melhoria na interface da agenda com calendário. - Trava no banco contra conflito de horários (Dia Inteiro vs Manhã/Tarde). - Funcionalidade de excluir agendamento ao arrastar para "Disponíveis". - Criação do botão de Upload da planilha de Estoque no Painel Web.
</commit_message>
<xml_diff>
--- a/data/banco_solicitacoes.xlsx
+++ b/data/banco_solicitacoes.xlsx
@@ -35,8 +35,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
   <fonts count="1">
@@ -401,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -671,19 +670,19 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B8" t="str">
-        <v>FINALIZADO</v>
+        <v>PENDENTE</v>
       </c>
       <c r="C8" t="str">
-        <v>18/07/2026, 13:56:49</v>
+        <v>19/07/2026, 21:22:29</v>
       </c>
       <c r="D8" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E8" t="str">
-        <v>PRINTI</v>
+        <v>ATUALCARD</v>
       </c>
       <c r="F8" t="str">
         <v>HP 12K - CIF</v>
@@ -698,10 +697,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J8" t="str">
-        <v>CT990-04870</v>
+        <v>CU498-04180</v>
       </c>
       <c r="K8" t="str">
-        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
+        <v>TAMPA DO FUSO</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -709,22 +708,22 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B9" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C9" t="str">
-        <v>18/07/2026, 13:56:16</v>
+        <v>18/07/2026, 13:56:49</v>
       </c>
       <c r="D9" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E9" t="str">
-        <v>ALPHA COLOR</v>
+        <v>PRINTI</v>
       </c>
       <c r="F9" t="str">
-        <v>HP WS6800 - CAREPACK</v>
+        <v>HP 12K - CIF</v>
       </c>
       <c r="G9" t="str">
         <v>Não</v>
@@ -736,10 +735,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J9" t="str">
-        <v>CU498-01813</v>
+        <v>CT990-04870</v>
       </c>
       <c r="K9" t="str">
-        <v>PLACA CONTROLADORA DE TRANSFERENCIA</v>
+        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
       </c>
       <c r="L9">
         <v>1</v>
@@ -774,10 +773,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J10" t="str">
-        <v>CT345-00746</v>
+        <v>CU498-01813</v>
       </c>
       <c r="K10" t="str">
-        <v>ROLO DE BORRACHA</v>
+        <v>PLACA CONTROLADORA DE TRANSFERENCIA</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -785,37 +784,37 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B11" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C11" t="str">
-        <v>18/07/2026, 13:38:07</v>
+        <v>18/07/2026, 13:56:16</v>
       </c>
       <c r="D11" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E11" t="str">
-        <v>PRINTI</v>
+        <v>ALPHA COLOR</v>
       </c>
       <c r="F11" t="str">
-        <v>HP 12K - CIF</v>
+        <v>HP WS6800 - CAREPACK</v>
       </c>
       <c r="G11" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="H11" t="str">
         <v>Atender</v>
       </c>
       <c r="I11" t="str">
-        <v>Prioridade MD</v>
+        <v>Atendimento Imediato</v>
       </c>
       <c r="J11" t="str">
-        <v>CT990-04870</v>
+        <v>CT345-00746</v>
       </c>
       <c r="K11" t="str">
-        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
+        <v>ROLO DE BORRACHA</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -823,13 +822,13 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C12" t="str">
-        <v>18/07/2026, 13:00:40</v>
+        <v>18/07/2026, 13:38:07</v>
       </c>
       <c r="D12" t="str">
         <v>MESTRE</v>
@@ -861,40 +860,40 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B13" t="str">
-        <v>REPROVADO</v>
+        <v>FINALIZADO</v>
       </c>
       <c r="C13" t="str">
-        <v>16/07/2026, 15:05:53</v>
+        <v>18/07/2026, 13:00:40</v>
       </c>
       <c r="D13" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E13" t="str">
-        <v>SERITEC</v>
+        <v>PRINTI</v>
       </c>
       <c r="F13" t="str">
-        <v>HP WS6800 - CAREPACK</v>
+        <v>HP 12K - CIF</v>
       </c>
       <c r="G13" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H13" t="str">
         <v>Atender</v>
       </c>
       <c r="I13" t="str">
-        <v>Atendimento Imediato</v>
+        <v>Prioridade MD</v>
       </c>
       <c r="J13" t="str">
-        <v>7000-09270</v>
+        <v>CT990-04870</v>
       </c>
       <c r="K13" t="str">
-        <v>ENGATE DE TRACAO DO ANILOX</v>
+        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -926,48 +925,48 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J14" t="str">
-        <v>7000-A14084-350</v>
+        <v>7000-09270</v>
       </c>
       <c r="K14" t="str">
-        <v>BANDEJA DE TINTA SEM DRENO</v>
+        <v>ENGATE DE TRACAO DO ANILOX</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" t="str">
-        <v>APROVADO</v>
+        <v>REPROVADO</v>
       </c>
       <c r="C15" t="str">
-        <v>16/07/2026, 10:06:46</v>
+        <v>16/07/2026, 15:05:53</v>
       </c>
       <c r="D15" t="str">
-        <v>ZANELLA</v>
+        <v>MESTRE</v>
       </c>
       <c r="E15" t="str">
-        <v>MEGA LABEL</v>
+        <v>SERITEC</v>
       </c>
       <c r="F15" t="str">
-        <v>HP 6K - VENDA</v>
+        <v>HP WS6800 - CAREPACK</v>
       </c>
       <c r="G15" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="H15" t="str">
         <v>Atender</v>
       </c>
       <c r="I15" t="str">
-        <v>Prioridade MD</v>
+        <v>Atendimento Imediato</v>
       </c>
       <c r="J15" t="str">
-        <v>CU150-01512</v>
+        <v>7000-A14084-350</v>
       </c>
       <c r="K15" t="str">
-        <v>CORREIA DO VENTILADOR</v>
+        <v>BANDEJA DE TINTA SEM DRENO</v>
       </c>
       <c r="L15">
         <v>1</v>
@@ -975,37 +974,37 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" t="str">
-        <v>FINALIZADO</v>
+        <v>APROVADO</v>
       </c>
       <c r="C16" t="str">
-        <v>15/07/2026, 16:17:05</v>
+        <v>16/07/2026, 10:06:46</v>
       </c>
       <c r="D16" t="str">
         <v>ZANELLA</v>
       </c>
       <c r="E16" t="str">
-        <v>PRINTI</v>
+        <v>MEGA LABEL</v>
       </c>
       <c r="F16" t="str">
-        <v>HP 12K - CIF</v>
+        <v>HP 6K - VENDA</v>
       </c>
       <c r="G16" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H16" t="str">
         <v>Atender</v>
       </c>
       <c r="I16" t="str">
-        <v>Atendimento Imediato</v>
+        <v>Prioridade MD</v>
       </c>
       <c r="J16" t="str">
-        <v>CU139-01483</v>
+        <v>CU150-01512</v>
       </c>
       <c r="K16" t="str">
-        <v>ATUADOR DE PORTA</v>
+        <v>CORREIA DO VENTILADOR</v>
       </c>
       <c r="L16">
         <v>1</v>
@@ -1013,22 +1012,22 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B17" t="str">
-        <v>REPROVADO</v>
+        <v>FINALIZADO</v>
       </c>
       <c r="C17" t="str">
-        <v>15/07/2026, 14:51:37</v>
+        <v>15/07/2026, 16:17:05</v>
       </c>
       <c r="D17" t="str">
         <v>ZANELLA</v>
       </c>
       <c r="E17" t="str">
-        <v>HELLOGRAF</v>
+        <v>PRINTI</v>
       </c>
       <c r="F17" t="str">
-        <v>HP 10K - VENDA</v>
+        <v>HP 12K - CIF</v>
       </c>
       <c r="G17" t="str">
         <v>Não</v>
@@ -1040,10 +1039,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J17" t="str">
-        <v>CT455-00370</v>
+        <v>CU139-01483</v>
       </c>
       <c r="K17" t="str">
-        <v>PLACA CONTROLADORA DO TANK DE TINTA ITSB</v>
+        <v>ATUADOR DE PORTA</v>
       </c>
       <c r="L17">
         <v>1</v>
@@ -1051,13 +1050,13 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B18" t="str">
-        <v>APROVADO</v>
+        <v>REPROVADO</v>
       </c>
       <c r="C18" t="str">
-        <v>14/07/2026, 17:32:56</v>
+        <v>15/07/2026, 14:51:37</v>
       </c>
       <c r="D18" t="str">
         <v>ZANELLA</v>
@@ -1069,19 +1068,19 @@
         <v>HP 10K - VENDA</v>
       </c>
       <c r="G18" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="H18" t="str">
         <v>Atender</v>
       </c>
       <c r="I18" t="str">
-        <v>Prioridade MD</v>
+        <v>Atendimento Imediato</v>
       </c>
       <c r="J18" t="str">
-        <v>CT990-03460</v>
+        <v>CT455-00370</v>
       </c>
       <c r="K18" t="str">
-        <v>CONEXAO 1/4M X 1/4M L38</v>
+        <v>PLACA CONTROLADORA DO TANK DE TINTA ITSB</v>
       </c>
       <c r="L18">
         <v>1</v>
@@ -1089,37 +1088,37 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B19" t="str">
-        <v>FINALIZADO</v>
+        <v>APROVADO</v>
       </c>
       <c r="C19" t="str">
-        <v>14/07/2026, 12:09:02</v>
+        <v>14/07/2026, 17:32:56</v>
       </c>
       <c r="D19" t="str">
         <v>ZANELLA</v>
       </c>
       <c r="E19" t="str">
-        <v>CAMARGO</v>
+        <v>HELLOGRAF</v>
       </c>
       <c r="F19" t="str">
-        <v>HP2 20K - CIF</v>
+        <v>HP 10K - VENDA</v>
       </c>
       <c r="G19" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H19" t="str">
         <v>Atender</v>
       </c>
       <c r="I19" t="str">
-        <v>UTK</v>
+        <v>Prioridade MD</v>
       </c>
       <c r="J19" t="str">
-        <v>CU010-03336</v>
+        <v>CT990-03460</v>
       </c>
       <c r="K19" t="str">
-        <v>VALVULA SOLENOIDE</v>
+        <v>CONEXAO 1/4M X 1/4M L38</v>
       </c>
       <c r="L19">
         <v>1</v>
@@ -1127,22 +1126,22 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B20" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C20" t="str">
-        <v>14/07/2026, 10:31:27</v>
+        <v>14/07/2026, 12:09:02</v>
       </c>
       <c r="D20" t="str">
         <v>ZANELLA</v>
       </c>
       <c r="E20" t="str">
-        <v>FORMA CERTA</v>
+        <v>CAMARGO</v>
       </c>
       <c r="F20" t="str">
-        <v>HP 100K - CIF</v>
+        <v>HP2 20K - CIF</v>
       </c>
       <c r="G20" t="str">
         <v>Não</v>
@@ -1151,13 +1150,13 @@
         <v>Atender</v>
       </c>
       <c r="I20" t="str">
-        <v>Atendimento Imediato</v>
+        <v>UTK</v>
       </c>
       <c r="J20" t="str">
-        <v>CT445-66660</v>
+        <v>CU010-03336</v>
       </c>
       <c r="K20" t="str">
-        <v>ROLETE</v>
+        <v>VALVULA SOLENOIDE</v>
       </c>
       <c r="L20">
         <v>1</v>
@@ -1192,13 +1191,13 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J21" t="str">
-        <v>CT445-25742</v>
+        <v>CT445-66660</v>
       </c>
       <c r="K21" t="str">
-        <v>ROLO DE TRACIONAMENTO DE PAPEL</v>
+        <v>ROLETE</v>
       </c>
       <c r="L21">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1230,56 +1229,94 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J22" t="str">
-        <v>CU153-02488</v>
+        <v>CT445-25742</v>
       </c>
       <c r="K22" t="str">
-        <v>MOLA DE GAS 300N 60ST K</v>
+        <v>ROLO DE TRACIONAMENTO DE PAPEL</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B23" t="str">
-        <v>IMPORTACAO</v>
+        <v>FINALIZADO</v>
       </c>
       <c r="C23" t="str">
-        <v>14/07/2026, 10:01:36</v>
+        <v>14/07/2026, 10:31:27</v>
       </c>
       <c r="D23" t="str">
         <v>ZANELLA</v>
       </c>
       <c r="E23" t="str">
+        <v>FORMA CERTA</v>
+      </c>
+      <c r="F23" t="str">
+        <v>HP 100K - CIF</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Atender</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Atendimento Imediato</v>
+      </c>
+      <c r="J23" t="str">
+        <v>CU153-02488</v>
+      </c>
+      <c r="K23" t="str">
+        <v>MOLA DE GAS 300N 60ST K</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>62</v>
+      </c>
+      <c r="B24" t="str">
+        <v>IMPORTACAO</v>
+      </c>
+      <c r="C24" t="str">
+        <v>14/07/2026, 10:01:36</v>
+      </c>
+      <c r="D24" t="str">
+        <v>ZANELLA</v>
+      </c>
+      <c r="E24" t="str">
         <v>PRINTI</v>
       </c>
-      <c r="F23" t="str">
+      <c r="F24" t="str">
         <v>HP 120K - CIF</v>
       </c>
-      <c r="G23" t="str">
-        <v>Não</v>
-      </c>
-      <c r="H23" t="str">
-        <v>Atender</v>
-      </c>
-      <c r="I23" t="str">
+      <c r="G24" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Atender</v>
+      </c>
+      <c r="I24" t="str">
         <v>UTK</v>
       </c>
-      <c r="J23" t="str">
+      <c r="J24" t="str">
         <v>CT001-77720</v>
       </c>
-      <c r="K23" t="str">
+      <c r="K24" t="str">
         <v>Importar</v>
       </c>
-      <c r="L23">
+      <c r="L24">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1563,7 +1600,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1605,19 +1642,19 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" t="str">
-        <v>FINALIZADO</v>
+        <v>PENDENTE</v>
       </c>
       <c r="C2" t="str">
-        <v>18/07/2026, 13:56:49</v>
+        <v>19/07/2026, 21:22:29</v>
       </c>
       <c r="D2" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E2" t="str">
-        <v>PRINTI</v>
+        <v>ATUALCARD</v>
       </c>
       <c r="F2" t="str">
         <v>HP 12K - CIF</v>
@@ -1632,10 +1669,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J2" t="str">
-        <v>CT990-04870</v>
+        <v>CU498-04180</v>
       </c>
       <c r="K2" t="str">
-        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
+        <v>TAMPA DO FUSO</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -1643,22 +1680,22 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B3" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C3" t="str">
-        <v>18/07/2026, 13:56:16</v>
+        <v>18/07/2026, 13:56:49</v>
       </c>
       <c r="D3" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E3" t="str">
-        <v>ALPHA COLOR</v>
+        <v>PRINTI</v>
       </c>
       <c r="F3" t="str">
-        <v>HP WS6800 - CAREPACK</v>
+        <v>HP 12K - CIF</v>
       </c>
       <c r="G3" t="str">
         <v>Não</v>
@@ -1670,10 +1707,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J3" t="str">
-        <v>CU498-01813</v>
+        <v>CT990-04870</v>
       </c>
       <c r="K3" t="str">
-        <v>PLACA CONTROLADORA DE TRANSFERENCIA</v>
+        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
       </c>
       <c r="L3">
         <v>1</v>
@@ -1708,10 +1745,10 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J4" t="str">
-        <v>CT345-00746</v>
+        <v>CU498-01813</v>
       </c>
       <c r="K4" t="str">
-        <v>ROLO DE BORRACHA</v>
+        <v>PLACA CONTROLADORA DE TRANSFERENCIA</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -1719,37 +1756,37 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C5" t="str">
-        <v>18/07/2026, 13:38:07</v>
+        <v>18/07/2026, 13:56:16</v>
       </c>
       <c r="D5" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E5" t="str">
-        <v>PRINTI</v>
+        <v>ALPHA COLOR</v>
       </c>
       <c r="F5" t="str">
-        <v>HP 12K - CIF</v>
+        <v>HP WS6800 - CAREPACK</v>
       </c>
       <c r="G5" t="str">
-        <v>Sim</v>
+        <v>Não</v>
       </c>
       <c r="H5" t="str">
         <v>Atender</v>
       </c>
       <c r="I5" t="str">
-        <v>Prioridade MD</v>
+        <v>Atendimento Imediato</v>
       </c>
       <c r="J5" t="str">
-        <v>CT990-04870</v>
+        <v>CT345-00746</v>
       </c>
       <c r="K5" t="str">
-        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
+        <v>ROLO DE BORRACHA</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -1757,13 +1794,13 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B6" t="str">
         <v>FINALIZADO</v>
       </c>
       <c r="C6" t="str">
-        <v>18/07/2026, 13:00:40</v>
+        <v>18/07/2026, 13:38:07</v>
       </c>
       <c r="D6" t="str">
         <v>MESTRE</v>
@@ -1795,40 +1832,40 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B7" t="str">
-        <v>REPROVADO</v>
+        <v>FINALIZADO</v>
       </c>
       <c r="C7" t="str">
-        <v>16/07/2026, 15:05:53</v>
+        <v>18/07/2026, 13:00:40</v>
       </c>
       <c r="D7" t="str">
         <v>MESTRE</v>
       </c>
       <c r="E7" t="str">
-        <v>SERITEC</v>
+        <v>PRINTI</v>
       </c>
       <c r="F7" t="str">
-        <v>HP WS6800 - CAREPACK</v>
+        <v>HP 12K - CIF</v>
       </c>
       <c r="G7" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H7" t="str">
         <v>Atender</v>
       </c>
       <c r="I7" t="str">
-        <v>Atendimento Imediato</v>
+        <v>Prioridade MD</v>
       </c>
       <c r="J7" t="str">
-        <v>7000-09270</v>
+        <v>CT990-04870</v>
       </c>
       <c r="K7" t="str">
-        <v>ENGATE DE TRACAO DO ANILOX</v>
+        <v>KIT DE PRIMEIRA TROCA DO NOVO VENTILADOR</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1860,18 +1897,56 @@
         <v>Atendimento Imediato</v>
       </c>
       <c r="J8" t="str">
+        <v>7000-09270</v>
+      </c>
+      <c r="K8" t="str">
+        <v>ENGATE DE TRACAO DO ANILOX</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>72</v>
+      </c>
+      <c r="B9" t="str">
+        <v>REPROVADO</v>
+      </c>
+      <c r="C9" t="str">
+        <v>16/07/2026, 15:05:53</v>
+      </c>
+      <c r="D9" t="str">
+        <v>MESTRE</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SERITEC</v>
+      </c>
+      <c r="F9" t="str">
+        <v>HP WS6800 - CAREPACK</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Atender</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Atendimento Imediato</v>
+      </c>
+      <c r="J9" t="str">
         <v>7000-A14084-350</v>
       </c>
-      <c r="K8" t="str">
+      <c r="K9" t="str">
         <v>BANDEJA DE TINTA SEM DRENO</v>
       </c>
-      <c r="L8">
+      <c r="L9">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>